<commit_message>
NumericType 改为通过 Luban 生成；Unit 表添加 Numeric 字段，添加 vba 表格函数 NumericRange。
</commit_message>
<xml_diff>
--- a/Unity/Assets/Config/Excel/__tables__.xlsx
+++ b/Unity/Assets/Config/Excel/__tables__.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27425"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Unity\ET8-Luban\Unity\Assets\Config\Excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\1_Code\UnityProject\ET\YIUI\Unity\Assets\Config\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E31600F-19BB-4EA8-934A-05CBB7D31578}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A175866D-884A-4BF6-99A6-F6438340CC15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7005" yWindow="2235" windowWidth="20460" windowHeight="11835" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -130,10 +130,6 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>UnitConfig.xlsx</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>资源配置</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -143,6 +139,10 @@
   </si>
   <si>
     <t>取值c|s，可以有多个，以逗号','分隔；空则表示属于所有分组；为了支持机器人运行，此项目里c代表c和s, s代表仅s。</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>UnitConfig.xlsm</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -556,7 +556,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="I1" s="3" t="s">
         <v>6</v>
@@ -620,7 +620,7 @@
         <v>21</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="I3" s="3"/>
       <c r="J3" s="3"/>
@@ -668,7 +668,7 @@
         <v>1</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="F5" s="1"/>
       <c r="G5" s="1"/>
@@ -700,7 +700,7 @@
       <c r="G6" s="1"/>
       <c r="H6" s="1"/>
       <c r="I6" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="J6" s="1"/>
       <c r="K6" s="1" t="str">

</xml_diff>